<commit_message>
Phase 4 follow-up: like-for-like reconciliation, planted discrepancies, rollups
- Catalogue: derived.counts / like_for_like per indicator; WASH-01 derived
  from people served on activity records; aggregation field on every
  indicator (sum / latest / average / ratio; WASH-04 latest until confirmed)
- indicators.py: monthly values rolled up by the aggregation method;
  partial targets keep "target incomplete" with partial % achieved and
  "partial: n of m months"; month-by-month reconciliation
- Generator: WASH-01 and AGR-01 reports from the same truth as activity and
  register data, with planted over-, under-reporting and rounding logged in
  the ground truth; main fingerprint c43d0b4d...; held-out sets unchanged
- Scorecard: reconciliation scoring (60/60 planted caught, 0 unexplained
  false alarms, 5/5 rounding within tolerance); third scorer correction
  (USD amounts) logged with evidence
- 263 tests passing

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/indicator_reference_sheets.xlsx
+++ b/docs/indicator_reference_sheets.xlsx
@@ -628,12 +628,12 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Reported: the sum of the monthly values in the indicator reports. Derived: the number of different registered people who received a "water point access" service (activity ACT01) during the period.</t>
+          <t>Reported: the sum of the monthly values in the indicator reports. Derived: the people served recorded in the activity records, i.e. the participants of water-point activities (activity ACT01) that took place during the month (completed or delayed), in the district where the activity took place.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Reported values are counts typed by officers and may include community members who are not registered. Derived values count each registered person once per period, however many services they received.</t>
+          <t>Both sources count people served by water-point activities as recorded by officers (not registered beneficiaries), so they are comparable. A person served by two water-point activities may be counted twice in both sources.</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>The two sources measure different things (all people reached versus registered beneficiaries), so a gap is expected; the reconciliation shows how large it is.</t>
+          <t>Reported and derived values are compared month by month in the reconciliation table; a gap above the tolerance points to a reporting or recording problem to follow up.</t>
         </is>
       </c>
       <c r="U3" s="4" t="inlineStr"/>
@@ -937,12 +937,12 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>The sum of the quarterly values in the indicator reports.</t>
+          <t>The latest quarterly value in the indicator reports for the period.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Each committee is counted once, in the quarter it is established. To be confirmed with partner whether the reports count NEW committees (which add up over a year, as calculated here) or ALL functional committees at the end of the quarter (which must not be added up).</t>
+          <t>Treated as a SNAPSHOT (aggregation: latest): a quarter or year shows the latest reported number of functional committees, not a sum. To be confirmed with partner whether the reports count new committees (which would add up, aggregation: sum) or all functional committees at the end of the quarter (as assumed here).</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Derived values count each registered person once per period, however many sessions they attended (not attendance). Reported values are counts typed by officers.</t>
+          <t>Each month counts different registered people (not attendance): a farmer at four sessions in one month counts once. Reported values are counts typed by officers for the same thing.</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>The definition of "trained" (one session, or the full course) needs to be agreed.</t>
+          <t>The definition of "trained" (one session, or the full course) needs to be agreed. Quarters and years add up the months, as the reports do, so a farmer trained in two different months counts in both.</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Phase 6: reconciliation levels, cost per person reached, annual pipeline gap, review, donor template
- Reconciliation level per indicator in the catalogue (WASH-01 district-month, AGR-01
  district-quarter, totals only; sex figures for information); scorer works at that level,
  lists planted discrepancies too small to detect, and runs for any set with planted ones
- CC-03 = activity cost / people reached as reported, by programme ("not available" when
  no reach is reported); new CC-05 cost per registered farmer trained (ACT10)
- Pipeline gap uses annual budgets (budget / project years); draft definition
- Donor template finished: donor dropdown from Donors sheet, percent probability,
  highlights, instructions and examples
- Review changes for the executive director, programme manager and MEAL officer
- Decision log D162-D167; screenshots retaken

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/indicator_reference_sheets.xlsx
+++ b/docs/indicator_reference_sheets.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Cost per beneficiary reached (RWF)</t>
+          <t>Cost per person reached (RWF), as reported</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1643,32 +1643,32 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Activity spending during the period divided by the number of different registered people reached.</t>
+          <t>Activity spending divided by the people reached as reported in the monthly indicator reports, by programme.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Total cost (RWF) of activities that took place during the period.</t>
+          <t>Total cost (RWF) of the activities of projects that report people reached, during the period.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Different registered people reached during the period.</t>
+          <t>People reached as reported by the same projects during the period: WASH programme - people with access to improved water (WASH-01); agriculture programme - farmers trained (AGR-01).</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Numerator divided by denominator.</t>
+          <t>Numerator divided by denominator. Not available for a project or programme that reports no reach.</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Unique people, not attendance. Costs are attributed to the district where the activity took place; people to the district where they registered.</t>
+          <t>Reported monthly figures are added up, as the reports do, so a person reached in two months counts twice. Projects without a people-reached indicator (sanitation, hygiene, irrigation) are left out of both sides.</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Activities with a cost recorded out of all activities that took place.</t>
+          <t>Activities whose cost is included (projects that report reach) out of all activities.</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>Activity monitoring files (costs) and beneficiary registers and service records (people) (derived).</t>
+          <t>Activity monitoring files (costs) and monthly indicator reports (people reached) (derived).</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>Only activity costs recorded in the monitoring files are included (not staff or overhead costs), and only registered people are counted, so the figure is not a full cost-effectiveness measure.</t>
+          <t>Replaces cost per REGISTERED person (D161, D163): the register holds far fewer people than the activities reach. Which indicators count "people reached" for each programme must be agreed with ARDE/KUBAHO; sanitation, hygiene and irrigation projects have none yet. Only activity costs are included (not staff or overheads).</t>
         </is>
       </c>
       <c r="U13" s="4" t="inlineStr"/>
@@ -1716,105 +1716,208 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>CC-05</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Cost per registered farmer trained, farmer field schools (RWF)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Draft, for co-design with ARDE/KUBAHO staff</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>RWF</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Cost of farmer field school sessions divided by the different registered people who attended them (training activities only).</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Total cost (RWF) of farmer field school sessions (ACT10) during the period.</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Different registered people who received farmer training (ACT10) during the period.</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Numerator divided by denominator.</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Unique people, not attendance. Training is the one activity where every participant is registered.</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Sessions with a cost recorded out of all sessions that took place.</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>To be agreed with ARDE/KUBAHO.</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>Activity monitoring files (costs) and beneficiary registers and service records (people) (derived).</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>To be confirmed with partner (suggested - finance officer with MEAL officer)</t>
+        </is>
+      </c>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>Kept for training activities only, where registration is complete; labelled as per REGISTERED farmer.</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>CC-04</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Reporting completeness: percentage of expected monthly reports submitted</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Draft, for co-design with ARDE/KUBAHO staff</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Cross-cutting</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Of the monthly indicator reports due, the percentage received.</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Reports received.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Reports due: one per project, district and month in which at least one of the project's indicators is due.</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Numerator divided by denominator, times 100.</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>One report per project, district and month.</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Not applicable (all expected reports are counted).</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>To be agreed with ARDE/KUBAHO (for example 100%).</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>Monthly indicator reports compared with the reporting schedule (derived).</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>available</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr">
+      <c r="R15" s="4" t="inlineStr">
         <is>
           <t>To be confirmed with partner (suggested - MEAL officer)</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
+      <c r="S15" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="T15" s="4" t="inlineStr">
         <is>
           <t>Uses the same definition as the "reporting completeness" data-quality measure (config/dq_metrics.yaml), so the two always agree.</t>
         </is>
       </c>
-      <c r="U14" s="4" t="inlineStr"/>
+      <c r="U15" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>